<commit_message>
Improve WebMCP activity and messaging flow
</commit_message>
<xml_diff>
--- a/assets/data/marktplaats_acoustic_guitars_emotional_seller_descriptions.xlsx
+++ b/assets/data/marktplaats_acoustic_guitars_emotional_seller_descriptions.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acoustic guitar listings" sheetId="1" r:id="Rc5d8cf7d47274b5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="2" r:id="Re8ba776984e54e03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acoustic guitar listings" sheetId="1" r:id="Reeec010361ea4ecb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="2" r:id="Rd71c7f0da1434db3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -337,7 +337,7 @@
         <x:v>Price</x:v>
       </x:c>
       <x:c r="C1" s="5" t="str">
-        <x:v>Image links</x:v>
+        <x:v>Image links removed</x:v>
       </x:c>
       <x:c r="D1" s="5" t="str">
         <x:v>Additional info</x:v>
@@ -349,7 +349,7 @@
         <x:v>Description source</x:v>
       </x:c>
       <x:c r="G1" s="5" t="str">
-        <x:v>Listing URL</x:v>
+        <x:v>Listing URL removed</x:v>
       </x:c>
       <x:c r="H1" s="10" t="str">
         <x:v>Seller tone</x:v>
@@ -368,9 +368,7 @@
       <x:c r="B2" s="14" t="str">
         <x:v>€ 1.699,-</x:v>
       </x:c>
-      <x:c r="C2" s="14" t="str">
-        <x:v>https://images.marktplaats.com/api/v1/hz-mp-pro-listing/images/43169ffb-d561-48ad-a21e-fba4d2d0b0da?rule=ecg_mp_eps%24_85</x:v>
-      </x:c>
+      <x:c r="C2" s="14" t="str"/>
       <x:c r="D2" s="14" t="str">
         <x:v>2009 · Furch G23-CR · Grand Auditorium · Solid Western Red Cedar top · Solid Indian Rosewood back/sides · Ebony fingerboard/bridge · Hiscox flightcase · Like new</x:v>
       </x:c>
@@ -378,11 +376,9 @@
         <x:v>A 2009 Furch G23-CR from the former Millennium series, described as being in exceptional condition. It has a solid Western Red Cedar top, solid Indian rosewood back and sides, ebony fingerboard and bridge, 45 mm nut width and gold Schaller tuners. The guitar has been carefully stored in its case and comes with the original heavy-duty Hiscox flightcase. The seller also offers an Acus acoustic amplifier separately or as a discounted bundle.</x:v>
       </x:c>
       <x:c r="F2" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G2" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/m2435922342-furch-g23-cr-2009-perfecte-staat-incl-hiscox-koffer</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G2" s="14" t="str"/>
       <x:c r="H2" s="14" t="str">
         <x:v>Urgent enthusiast / meticulous</x:v>
       </x:c>
@@ -400,9 +396,7 @@
       <x:c r="B3" s="14" t="str">
         <x:v>€ 100,-</x:v>
       </x:c>
-      <x:c r="C3" s="14" t="str">
-        <x:v>https://images.marktplaats.com/api/v1/hz-mp-pro-listing/images/53e76882-76ea-43f0-bb61-6bba13af52bf?rule=ecg_mp_eps%24_85</x:v>
-      </x:c>
+      <x:c r="C3" s="14" t="str"/>
       <x:c r="D3" s="14" t="str">
         <x:v>1973 · Sigma DR-7 · First generation · Made in Japan for Martin · Rosewood · Handwritten serial · Used / visibly aged</x:v>
       </x:c>
@@ -410,11 +404,9 @@
         <x:v>A first-generation 1973 Sigma DR-7, one of the early Japanese-made Sigma instruments produced for Martin with US quality control. It still has a handwritten serial number and rosewood construction. The seller is thinning a collection and is candid that the guitar has clearly lived a life and needs some care, but says it still sounds excellent and can be tried in Apeldoorn.</x:v>
       </x:c>
       <x:c r="F3" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G3" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/m2435476812-vintage-sigma-dr-7-made-in-japan</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G3" s="14" t="str"/>
       <x:c r="H3" s="14" t="str">
         <x:v>Nostalgic collector / affectionate</x:v>
       </x:c>
@@ -432,9 +424,7 @@
       <x:c r="B4" s="14" t="str">
         <x:v>€ 3.750,-</x:v>
       </x:c>
-      <x:c r="C4" s="14" t="str">
-        <x:v>https://images.marktplaats.com/api/v1/hz-mp-pro-listing/images/28df3a89-3402-4127-9e9b-9de00a55130e?rule=ecg_mp_eps%24_85</x:v>
-      </x:c>
+      <x:c r="C4" s="14" t="str"/>
       <x:c r="D4" s="14" t="str">
         <x:v>2021 · Martin HD-35 Reimagined · Dreadnought · Like new · Case included · Carefully maintained</x:v>
       </x:c>
@@ -442,11 +432,9 @@
         <x:v>A 2021 Martin HD-35 Reimagined presented in near-new condition. The seller describes it as a high-end dreadnought for a discerning player, carefully maintained and rarely removed from its case. The HD-35 is highlighted for its deep, room-filling sound and refined response, and the original case is included.</x:v>
       </x:c>
       <x:c r="F4" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G4" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/m2435780485-martin-hd-35-reimagined-2021-nieuwstaat</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G4" s="14" t="str"/>
       <x:c r="H4" s="14" t="str">
         <x:v>Proud / reluctant connoisseur</x:v>
       </x:c>
@@ -464,9 +452,7 @@
       <x:c r="B5" s="14" t="str">
         <x:v>€ 250,-</x:v>
       </x:c>
-      <x:c r="C5" s="14" t="str">
-        <x:v>https://images.marktplaats.com/api/v1/hz-mp-pro-listing/images/167b7f1f-42b1-4608-9f95-fed1a71cb0f9?rule=ecg_mp_eps%24_85</x:v>
-      </x:c>
+      <x:c r="C5" s="14" t="str"/>
       <x:c r="D5" s="14" t="str">
         <x:v>Purchased 1993 · Sigma DM-2 · Mahogany · Made in Korea · Sigma by Martin · Recently set up by local luthier · Used</x:v>
       </x:c>
@@ -474,11 +460,9 @@
         <x:v>A Sigma DM-2 mahogany acoustic bought in Amersfoort in 1993 and built in Korea as a third-generation Sigma by Martin. It was professionally set up by a local luthier a few years ago and is said to play comfortably with a pleasant tone. It shows normal age-related wear but no serious damage. The seller is reducing a personal collection.</x:v>
       </x:c>
       <x:c r="F5" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G5" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/m2435503058-mooie-sigma-dm-2-gitaar-made-in-korea</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G5" s="14" t="str"/>
       <x:c r="H5" s="14" t="str">
         <x:v>Warm collector / practical</x:v>
       </x:c>
@@ -496,9 +480,7 @@
       <x:c r="B6" s="14" t="str">
         <x:v>€ 6.875,-</x:v>
       </x:c>
-      <x:c r="C6" s="14" t="str">
-        <x:v>https://images.marktplaats.com/api/v1/hz-mp-pro-listing/images/f9a6da80-dd8f-4565-889c-5564c3691e6a?rule=ecg_mp_eps%24_85</x:v>
-      </x:c>
+      <x:c r="C6" s="14" t="str"/>
       <x:c r="D6" s="14" t="str">
         <x:v>2026 · Martin D-42 Modern Deluxe · Played about 4 times · Original case · Purchased 27-03-2026 at TFOA · Warranty remaining</x:v>
       </x:c>
@@ -506,11 +488,9 @@
         <x:v>An almost-new Martin D-42 Modern Deluxe purchased from The Fellowship of Acoustics on 27 March 2026 and reportedly played only four times. It remains under warranty and comes with its original case. The seller describes it as a premium western guitar with rich tone and excellent playability, effectively offering a nearly new instrument at a used-market price.</x:v>
       </x:c>
       <x:c r="F6" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G6" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/m2435475420-martin-d-42-modern-deluxe-nieuwstaat-aankoop-maart-2026</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G6" s="14" t="str"/>
       <x:c r="H6" s="14" t="str">
         <x:v>Excited / premium opportunity</x:v>
       </x:c>
@@ -528,9 +508,7 @@
       <x:c r="B7" s="14" t="str">
         <x:v>€ 700,-</x:v>
       </x:c>
-      <x:c r="C7" s="14" t="str">
-        <x:v>https://images.marktplaats.com/api/v1/hz-mp-pro-listing/images/b8226576-af73-4796-be37-42ab2b530d13?rule=ecg_mp_eps%24_85</x:v>
-      </x:c>
+      <x:c r="C7" s="14" t="str"/>
       <x:c r="D7" s="14" t="str">
         <x:v>2007 · Alhambra 7P · Classical Spanish guitar · Solid spruce top · Made in Spain · Case included · Normal wear</x:v>
       </x:c>
@@ -538,11 +516,9 @@
         <x:v>A 2007 Alhambra 7P classical guitar from the brand's higher professional range, supplied with a case. It has a solid spruce top and is described as producing a clear, warm and dynamic sound with good projection. The seller emphasizes that almost two decades of playing and ageing have helped the solid top develop more depth and character. Normal age-related marks are present.</x:v>
       </x:c>
       <x:c r="F7" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G7" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/m2433330633-alhambra-7p-uit-2007-massief-sparren-bovenblad-inclusief</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G7" s="14" t="str"/>
       <x:c r="H7" s="14" t="str">
         <x:v>Thoughtful / tone-focused</x:v>
       </x:c>
@@ -560,9 +536,7 @@
       <x:c r="B8" s="14" t="str">
         <x:v>Bidding from € 675,-</x:v>
       </x:c>
-      <x:c r="C8" s="14" t="str">
-        <x:v>https://images.marktplaats.com/api/v1/hz-mp-pro-listing/images/f8c3c2c9-09d7-40ba-9ea0-1b608d8ba6e7?rule=ecg_mp_eps%24_85</x:v>
-      </x:c>
+      <x:c r="C8" s="14" t="str"/>
       <x:c r="D8" s="14" t="str">
         <x:v>2007 · Godin A6 Ultra · Hybrid acoustic/electric · Piezo + Godin humbucker · Dual outputs · Cedar top · Gigbag · Near mint</x:v>
       </x:c>
@@ -570,11 +544,9 @@
         <x:v>A 2007 Godin A6 Ultra hybrid acoustic/electric in exceptionally clean condition. The instrument combines an under-saddle piezo system for acoustic tones with a Godin neck humbucker for electric sounds, plus separate acoustic/mix and electric outputs. The seller says even the soft cedar top remains free from dents and scratches. The price has been reduced and bidding starts at €675.</x:v>
       </x:c>
       <x:c r="F8" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G8" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/m2431150854-godin-a6-ultra-gitaar-2007-zgan-gigbag</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G8" s="14" t="str"/>
       <x:c r="H8" s="14" t="str">
         <x:v>Proud / motivated</x:v>
       </x:c>
@@ -592,9 +564,7 @@
       <x:c r="B9" s="14" t="str">
         <x:v>€ 1.099,-</x:v>
       </x:c>
-      <x:c r="C9" s="14" t="str">
-        <x:v>https://admarkt-cdn.marktplaats.com/api/v1/icas-mp-pro-admarkt/images/92/92def5b9-e466-4a18-99b4-2da1e427aa7c?rule=eps_85</x:v>
-      </x:c>
+      <x:c r="C9" s="14" t="str"/>
       <x:c r="D9" s="14" t="str">
         <x:v>c.2000 · Larrivee OM-01 · Canada · OM body · Piezo pickup · Medium C neck · 25.5-inch scale · Case included · Excellent condition</x:v>
       </x:c>
@@ -602,11 +572,9 @@
         <x:v>A Canadian-made Larrivee OM-01 from around 2000 in natural finish. The shop describes it as a straightforward, well-built OM with a medium-C neck, 25.5-inch scale and piezo pickup for stage or studio use. Overall condition is excellent, with moderate fret wear appropriate to its age, and a case is included.</x:v>
       </x:c>
       <x:c r="F9" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G9" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/a1529038168-larrivee-om-01-ca-2000-natural</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G9" s="14" t="str"/>
       <x:c r="H9" s="14" t="str">
         <x:v>No-nonsense dealer</x:v>
       </x:c>
@@ -624,9 +592,7 @@
       <x:c r="B10" s="14" t="str">
         <x:v>Bidding</x:v>
       </x:c>
-      <x:c r="C10" s="14" t="str">
-        <x:v>https://images.marktplaats.com/api/v1/hz-mp-pro-listing/images/b687235e-cdf3-494a-bc81-8966ff082b5c?rule=ecg_mp_eps%24_85</x:v>
-      </x:c>
+      <x:c r="C10" s="14" t="str"/>
       <x:c r="D10" s="14" t="str">
         <x:v>Martinez ES10-S Sevilla · Classical guitar · Godoy Series · Solid spruce top · Mahogany back/sides · Like new</x:v>
       </x:c>
@@ -634,11 +600,9 @@
         <x:v>A Martinez ES10-S Sevilla classical guitar from the Godoy Series, presented in near-new condition. It uses a solid spruce top with mahogany back and sides, a combination described as producing a rich, warm tone with good resonance and a slight percussive character. The model is positioned for both developing and more experienced classical or flamenco players.</x:v>
       </x:c>
       <x:c r="F10" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G10" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/m2435102232-martinez-es10-s-sevilla</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G10" s="14" t="str"/>
       <x:c r="H10" s="14" t="str">
         <x:v>Enthusiastic / inviting</x:v>
       </x:c>
@@ -656,9 +620,7 @@
       <x:c r="B11" s="14" t="str">
         <x:v>€ 50,-</x:v>
       </x:c>
-      <x:c r="C11" s="14" t="str">
-        <x:v>https://images.marktplaats.com/api/v1/hz-mp-pro-listing/images/dabd7b37-ce01-4315-9f94-02da9a3d4478?rule=ecg_mp_eps%24_85</x:v>
-      </x:c>
+      <x:c r="C11" s="14" t="str"/>
       <x:c r="D11" s="14" t="str">
         <x:v>Morgan western guitar · Steel-string · Used · Warm tone · Comfortable action · Light cosmetic wear</x:v>
       </x:c>
@@ -666,11 +628,9 @@
         <x:v>A simple used Morgan western guitar offered as an affordable beginner instrument or second guitar. The seller describes it as comfortable to play with a warm acoustic tone. It has light age-related marks but remains in good functional condition and is suited to home practice or casual acoustic sessions.</x:v>
       </x:c>
       <x:c r="F11" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G11" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/m2435099412-morgan-western-gitaar-goede-staat</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G11" s="14" t="str"/>
       <x:c r="H11" s="14" t="str">
         <x:v>Casual / friendly</x:v>
       </x:c>
@@ -688,9 +648,7 @@
       <x:c r="B12" s="14" t="str">
         <x:v>€ 4.695,-</x:v>
       </x:c>
-      <x:c r="C12" s="14" t="str">
-        <x:v>https://admarkt-cdn.marktplaats.com/api/v1/icas-mp-pro-admarkt/images/3a/3ab3ba6d-e113-4be1-8afc-ac1b1384dc03?rule=eps_85</x:v>
-      </x:c>
+      <x:c r="C12" s="14" t="str"/>
       <x:c r="D12" s="14" t="str">
         <x:v>2019 · Lowden S-35W · UK-built · Figured walnut body · Cherry/walnut neck · 45 mm nut · Case · Excellent condition</x:v>
       </x:c>
@@ -698,11 +656,9 @@
         <x:v>A 2019 UK-built Lowden S-35W in a distinctive figured-walnut natural finish. It uses a walnut body with a cherry/walnut neck, 25.6-inch scale and 45 mm nut, giving extra space for chords and fingerstyle work. The guitar is in excellent condition and remains original except for one strap button. A case is included.</x:v>
       </x:c>
       <x:c r="F12" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G12" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/a1529873556-lowden-s-35w-2019-figured-walnut-natural</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G12" s="14" t="str"/>
       <x:c r="H12" s="14" t="str">
         <x:v>Boutique dealer / understated</x:v>
       </x:c>
@@ -715,26 +671,22 @@
     </x:row>
     <x:row r="13" ht="116" customHeight="1">
       <x:c r="A13" s="14" t="str">
-        <x:v>Diverse Western en klassieke gitaren vanaf €59,00 Emmen</x:v>
+        <x:v>Diverse Western en klassieke gitaren vanaf €59,00 the area</x:v>
       </x:c>
       <x:c r="B13" s="14" t="str">
         <x:v>From € 59,-</x:v>
       </x:c>
-      <x:c r="C13" s="14" t="str">
-        <x:v>https://images.marktplaats.com/api/v1/hz-mp-pro-listing/images/edbcb442-5ec0-40a2-ae59-35701191f923?rule=ecg_mp_eps%24_85</x:v>
-      </x:c>
+      <x:c r="C13" s="14" t="str"/>
       <x:c r="D13" s="14" t="str">
         <x:v>Mixed new/used collection · Classical, western, electro-acoustic and resonator guitars · Examples €59-€289+ · Pickup preferred</x:v>
       </x:c>
       <x:c r="E13" s="14" t="str">
-        <x:v>A private multi-guitar listing with a rotating mix of new, demo and used acoustic instruments. Examples include Recording King western guitars, a €59 Valencia classical, Nashville/Richwood electro-acoustics, a discounted Cort Luce demo, a Recording King resonator, Yamaha CX40 electro-acoustic and several budget western guitars. Pickup and testing in Emmen are preferred and may result in a sharper price, though shipping is also possible.</x:v>
+        <x:v>A private multi-guitar listing with a rotating mix of new, demo and used acoustic instruments. Examples include Recording King western guitars, a €59 Valencia classical, Nashville/Richwood electro-acoustics, a discounted Cort Luce demo, a Recording King resonator, Yamaha CX40 electro-acoustic and several budget western guitars. Pickup and testing in the area are preferred and may result in a sharper price, though shipping is also possible.</x:v>
       </x:c>
       <x:c r="F13" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G13" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/m2435090082-diverse-western-en-klassieke-gitaren-vanaf-59-00-emmen</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G13" s="14" t="str"/>
       <x:c r="H13" s="14" t="str">
         <x:v>Bargain-hunter / sociable</x:v>
       </x:c>
@@ -742,7 +694,7 @@
         <x:v>Flexible, especially on pickup</x:v>
       </x:c>
       <x:c r="J13" s="14" t="str">
-        <x:v>This is less one guitar and more my little acoustic-guitar corner of Emmen. There are classicals, westerns, electro-acoustics, demo instruments and even a resonator, starting at €59. I much prefer people to come over, try a few and hear the differences themselves. If you collect in person, I can often sharpen the price a bit too.</x:v>
+        <x:v>This is less one guitar and more my little acoustic-guitar corner of the area. There are classicals, westerns, electro-acoustics, demo instruments and even a resonator, starting at €59. I much prefer people to come over, try a few and hear the differences themselves. If you collect in person, I can often sharpen the price a bit too.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="116" customHeight="1">
@@ -752,9 +704,7 @@
       <x:c r="B14" s="14" t="str">
         <x:v>€ 2.995,-</x:v>
       </x:c>
-      <x:c r="C14" s="14" t="str">
-        <x:v>https://images.marktplaats.com/api/v1/hz-mp-pro-listing/images/75d6765f-d219-46f1-b263-5e786a691ca0?rule=ecg_mp_eps%24_85</x:v>
-      </x:c>
+      <x:c r="C14" s="14" t="str"/>
       <x:c r="D14" s="14" t="str">
         <x:v>Furch Orange OM-LG Limited Edition · Madagascar rosewood · Only 21 made worldwide · Fishman Ellipse Matrix Blend · Original case + certificate · Like new</x:v>
       </x:c>
@@ -762,11 +712,9 @@
         <x:v>A rare Furch Orange OM-LG Limited Edition in near-new condition, built with a Madagascar rosewood body. Only 21 examples were reportedly produced worldwide. It is equipped with a Fishman Ellipse Matrix Blend pickup/preamp and comes with the original case and authenticity certificate, making it attractive to both serious players and collectors.</x:v>
       </x:c>
       <x:c r="F14" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G14" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/m2427404869-furch-orange-om-lg-limited-edition-madagaskar-palissander</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G14" s="14" t="str"/>
       <x:c r="H14" s="14" t="str">
         <x:v>Collector pride / exclusive</x:v>
       </x:c>
@@ -779,26 +727,22 @@
     </x:row>
     <x:row r="15" ht="116" customHeight="1">
       <x:c r="A15" s="14" t="str">
-        <x:v>Lowden PB Pierre Bensusan Signature 2018 | Natural</x:v>
+        <x:v>Lowden PB Lucien Varo Signature 2018 | Natural</x:v>
       </x:c>
       <x:c r="B15" s="14" t="str">
         <x:v>€ 6.495,-</x:v>
       </x:c>
-      <x:c r="C15" s="14" t="str">
-        <x:v>https://admarkt-cdn.marktplaats.com/api/v1/icas-mp-pro-admarkt/images/28/2899d7bf-84dd-4e72-9afa-dfe169b9eda0?rule=eps_85</x:v>
-      </x:c>
+      <x:c r="C15" s="14" t="str"/>
       <x:c r="D15" s="14" t="str">
-        <x:v>2018 · Lowden Pierre Bensusan Signature · UK-built · 25.6-inch scale · 22 frets · Spruce/rosewood body · Maple neck · Ebony fingerboard · Case</x:v>
+        <x:v>2018 · Lowden Lucien Varo Signature · UK-built · 25.6-inch scale · 22 frets · Spruce/rosewood body · Maple neck · Ebony fingerboard · Case</x:v>
       </x:c>
       <x:c r="E15" s="14" t="str">
-        <x:v>A 2018 Lowden Pierre Bensusan Signature acoustic built in the UK. The signature model combines a 25.6-inch scale and 22 frets with a maple neck, ebony fingerboard and spruce/rosewood body. It is described as fully original and in excellent condition with a case included, aimed particularly at players seeking a distinctive high-end fingerstyle instrument.</x:v>
+        <x:v>A 2018 Lowden Lucien Varo Signature acoustic built in the UK. The signature model combines a 25.6-inch scale and 22 frets with a maple neck, ebony fingerboard and spruce/rosewood body. It is described as fully original and in excellent condition with a case included, aimed particularly at players seeking a distinctive high-end fingerstyle instrument.</x:v>
       </x:c>
       <x:c r="F15" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G15" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/a1529873558-lowden-pb-pierre-bensusan-signature-2018-natural</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G15" s="14" t="str"/>
       <x:c r="H15" s="14" t="str">
         <x:v>Connoisseur dealer</x:v>
       </x:c>
@@ -806,7 +750,7 @@
         <x:v>Premium dealer price</x:v>
       </x:c>
       <x:c r="J15" s="14" t="str">
-        <x:v>A Pierre Bensusan Signature Lowden is not really a generic 'nice acoustic'. It has its own geometry, feel and voice, designed around one of the defining modern fingerstyle players. This 2018 example is fully original, in excellent condition and comes with its case. If you already know why this model exists, the €6,495 price will make more sense than any amount of sales copy.</x:v>
+        <x:v>A Lucien Varo Signature Lowden is not really a generic 'nice acoustic'. It has its own geometry, feel and voice, designed around one of the defining modern fingerstyle players. This 2018 example is fully original, in excellent condition and comes with its case. If you already know why this model exists, the €6,495 price will make more sense than any amount of sales copy.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="116" customHeight="1">
@@ -816,9 +760,7 @@
       <x:c r="B16" s="14" t="str">
         <x:v>From € 150 each</x:v>
       </x:c>
-      <x:c r="C16" s="14" t="str">
-        <x:v>https://images.marktplaats.com/api/v1/hz-mp-pro-listing/images/722244d8-6846-4ac7-8d72-163919cae30d?rule=ecg_mp_eps%24_85</x:v>
-      </x:c>
+      <x:c r="C16" s="14" t="str"/>
       <x:c r="D16" s="14" t="str">
         <x:v>Ibanez V72ECE-NT + Tanglewood TW28DLX + Tanglewood TC3 · Used · Set up · Fresh D'Addario XS strings · Bags included on some · Trade possible</x:v>
       </x:c>
@@ -826,11 +768,9 @@
         <x:v>A small collection of used Ibanez and Tanglewood acoustics offered individually from €150. The guitars have been set up, fitted with fresh D'Addario XS Nano strings and are described as fully functional and in good condition. Some include bags. The seller is also open to trades, especially for several specific Tanglewood models with a preference for cutaway versions.</x:v>
       </x:c>
       <x:c r="F16" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G16" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/m2425449916-ibanez-v72ece-nt-tanglewood-tc3-tw28-gitaar-p-stk-150</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G16" s="14" t="str"/>
       <x:c r="H16" s="14" t="str">
         <x:v>Hobbyist / trade-friendly</x:v>
       </x:c>
@@ -848,9 +788,7 @@
       <x:c r="B17" s="14" t="str">
         <x:v>€ 975,-</x:v>
       </x:c>
-      <x:c r="C17" s="14" t="str">
-        <x:v>https://images.marktplaats.com/api/v1/hz-mp-pro-listing/images/4dbc1652-fb2a-4a30-bd87-d6ea78029349?rule=ecg_mp_eps%24_85</x:v>
-      </x:c>
+      <x:c r="C17" s="14" t="str"/>
       <x:c r="D17" s="14" t="str">
         <x:v>Eastman E6D-TC · All-solid dreadnought · Sitka spruce top · Mahogany body · Ebony bridge/fingerboard · Nitro finish · Eastman case + invoice · Like new</x:v>
       </x:c>
@@ -858,11 +796,9 @@
         <x:v>An Eastman E6D-TC all-solid dreadnought with Sitka spruce top and mahogany body. The bridge and fingerboard are ebony and the guitar uses a nitrocellulose finish usually found on more expensive instruments. The seller describes a warm, well-defined sound and says the guitar has seen very little use since being purchased new two years ago. The original Eastman case and invoice are included.</x:v>
       </x:c>
       <x:c r="F17" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G17" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/m2434687806-eastman-e6d-tc-dreadnought-gitaar</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G17" s="14" t="str"/>
       <x:c r="H17" s="14" t="str">
         <x:v>Proud / value-conscious</x:v>
       </x:c>
@@ -880,9 +816,7 @@
       <x:c r="B18" s="14" t="str">
         <x:v>€ 699,-</x:v>
       </x:c>
-      <x:c r="C18" s="14" t="str">
-        <x:v>https://admarkt-cdn.marktplaats.com/api/v1/icas-mp-pro-admarkt/images/cf/cf9e18c3-ec12-47df-b0fd-b10405441bea?rule=eps_85</x:v>
-      </x:c>
+      <x:c r="C18" s="14" t="str"/>
       <x:c r="D18" s="14" t="str">
         <x:v>2014 · Guild D-150 Westerly Collection · Dreadnought · Natural · 25.5-inch scale · Slim C neck · Rosewood fingerboard/bridge · Case · Excellent</x:v>
       </x:c>
@@ -890,11 +824,9 @@
         <x:v>A 2014 Guild D-150 Westerly Collection dreadnought in natural finish. The China-built model uses a 25.5-inch scale, slim-C neck and rosewood fingerboard and bridge. The dealer describes it as completely original, in excellent condition and supplied with a case, positioning it as a straightforward way into a traditional Guild-style dreadnought.</x:v>
       </x:c>
       <x:c r="F18" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G18" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/a1529500861-guild-d-150-westerly-collection-2014-natural</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G18" s="14" t="str"/>
       <x:c r="H18" s="14" t="str">
         <x:v>Straight dealer / no hype</x:v>
       </x:c>
@@ -907,26 +839,22 @@
     </x:row>
     <x:row r="19" ht="116" customHeight="1">
       <x:c r="A19" s="14" t="str">
-        <x:v>Martin D35 Johnny Cash (2013) met Sunrise pickup</x:v>
+        <x:v>Martin D35 Riley Cade (2013) met Sunrise pickup</x:v>
       </x:c>
       <x:c r="B19" s="14" t="str">
         <x:v>€ 5.250,-</x:v>
       </x:c>
-      <x:c r="C19" s="14" t="str">
-        <x:v>https://images.marktplaats.com/api/v1/hz-mp-pro-listing/images/064f3bff-cec1-4e57-b690-e7c5395648f0?rule=ecg_mp_eps%24_85</x:v>
-      </x:c>
+      <x:c r="C19" s="14" t="str"/>
       <x:c r="D19" s="14" t="str">
-        <x:v>2013 · Martin D-35 Johnny Cash · Sunrise pickup + preamp · Original-style black case · Professionally serviced · Small play wear · Binding professionally repaired</x:v>
+        <x:v>2013 · Martin D-35 Riley Cade · Sunrise pickup + preamp · Original-style black case · Professionally serviced · Small play wear · Binding professionally repaired</x:v>
       </x:c>
       <x:c r="E19" s="14" t="str">
-        <x:v>A 2013 Martin D-35 Johnny Cash edition in very good played condition. It has a removable Sunrise pickup with preamp, allowing high-quality amplified use without permanent modification. The seller notes small normal scratches and a professionally repaired section of binding, but says the frets, setup and overall condition are strong. It includes the black case and is praised for deep, warm projection across fingerstyle, strumming and flatpicking. Trades are not wanted unless it is a similarly valued Gibson J-45.</x:v>
+        <x:v>A 2013 Martin D-35 Riley Cade edition in very good played condition. It has a removable Sunrise pickup with preamp, allowing high-quality amplified use without permanent modification. The seller notes small normal scratches and a professionally repaired section of binding, but says the frets, setup and overall condition are strong. It includes the black case and is praised for deep, warm projection across fingerstyle, strumming and flatpicking. Trades are not wanted unless it is a similarly valued Gibson J-45.</x:v>
       </x:c>
       <x:c r="F19" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G19" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/m2434622593-martin-d35-johnny-cash-2013-met-sunrise-pickup</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G19" s="14" t="str"/>
       <x:c r="H19" s="14" t="str">
         <x:v>Fan / emotionally attached</x:v>
       </x:c>
@@ -944,9 +872,7 @@
       <x:c r="B20" s="14" t="str">
         <x:v>€ 1.500,-</x:v>
       </x:c>
-      <x:c r="C20" s="14" t="str">
-        <x:v>https://images.marktplaats.com/api/v1/hz-mp-pro-listing/images/8f47c621-527c-44d1-9e58-5842ddbc741c?rule=ecg_mp_eps%24_85</x:v>
-      </x:c>
+      <x:c r="C20" s="14" t="str"/>
       <x:c r="D20" s="14" t="str">
         <x:v>Taylor 414ce · Grand Auditorium · Cutaway · Piezo pickup · Solid Sitka spruce top · Solid ovangkol back/sides · Original case · Like new</x:v>
       </x:c>
@@ -954,11 +880,9 @@
         <x:v>A Taylor 414ce Grand Auditorium in near-new condition with original case. The guitar has a cutaway and onboard piezo pickup for stage use, with a solid Sitka spruce top and solid ovangkol back and sides. The seller highlights its balanced amplified tone and comfortable, versatile design for both studio and live playing. Offers are expected to reflect the instrument's value.</x:v>
       </x:c>
       <x:c r="F20" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G20" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/m2431658665-taylor-414ce-westerngitaar-met-koffer</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G20" s="14" t="str"/>
       <x:c r="H20" s="14" t="str">
         <x:v>Confident / polished</x:v>
       </x:c>
@@ -976,9 +900,7 @@
       <x:c r="B21" s="14" t="str">
         <x:v>€ 995,-</x:v>
       </x:c>
-      <x:c r="C21" s="14" t="str">
-        <x:v>https://images.marktplaats.com/api/v1/hz-mp-pro-listing/images/5026cca6-b890-48f3-90b8-022521bd2d37?rule=ecg_mp_eps%24_85</x:v>
-      </x:c>
+      <x:c r="C21" s="14" t="str"/>
       <x:c r="D21" s="14" t="str">
         <x:v>Taylor AD17e American Dream · USA-made · All-solid · Spruce top · Walnut back/sides · Mahogany neck · Eucalyptus fingerboard · Grand Pacific · Receipt included</x:v>
       </x:c>
@@ -986,11 +908,9 @@
         <x:v>A Taylor AD17e from the USA-made American Dream series, offered in good condition with only minimal normal signs of use. It uses all-solid construction, with a spruce top, walnut back and sides, mahogany neck and eucalyptus fingerboard. The Grand Pacific body has rounded shoulders and comfort-oriented edges, and the original purchase receipt is available. The seller states an original purchase price of €1,799.</x:v>
       </x:c>
       <x:c r="F21" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G21" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/m2432861792-taylor-ad17e-natural-top</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G21" s="14" t="str"/>
       <x:c r="H21" s="14" t="str">
         <x:v>Practical / value seller</x:v>
       </x:c>
@@ -1003,26 +923,22 @@
     </x:row>
     <x:row r="22" ht="116" customHeight="1">
       <x:c r="A22" s="14" t="str">
-        <x:v>Concertgitaar - Dominique Delarue</x:v>
+        <x:v>Concertgitaar - Celeste Maren</x:v>
       </x:c>
       <x:c r="B22" s="14" t="str">
         <x:v>€ 3.990,-</x:v>
       </x:c>
-      <x:c r="C22" s="14" t="str">
-        <x:v>https://images.marktplaats.com/api/v1/hz-mp-pro-listing/images/9ebfa39e-dce6-4626-b90c-1caca56be3d3?rule=ecg_mp_eps%24_85</x:v>
-      </x:c>
+      <x:c r="C22" s="14" t="str"/>
       <x:c r="D22" s="14" t="str">
-        <x:v>Dominique Delarue concert classical guitar · France · High-end luthier instrument · Case included · Like new</x:v>
+        <x:v>Celeste Maren concert classical guitar · France · High-end luthier instrument · Case included · Like new</x:v>
       </x:c>
       <x:c r="E22" s="14" t="str">
-        <x:v>A high-end concert classical guitar by French luthier Dominique Delarue. The listing presents Delarue as strongly influenced by Daniel Friederich and highly regarded among classical-guitar circles, with the instrument praised for a rich, refined voice. The guitar is offered in near-new condition with a case and is aimed at serious classical players rather than students looking for a basic instrument.</x:v>
+        <x:v>A high-end concert classical guitar by French luthier Celeste Maren. The listing presents Delarue as strongly influenced by Daniel Friederich and highly regarded among classical-guitar circles, with the instrument praised for a rich, refined voice. The guitar is offered in near-new condition with a case and is aimed at serious classical players rather than students looking for a basic instrument.</x:v>
       </x:c>
       <x:c r="F22" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G22" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/m2434354284-concertgitaar</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G22" s="14" t="str"/>
       <x:c r="H22" s="14" t="str">
         <x:v>Reverent / classical connoisseur</x:v>
       </x:c>
@@ -1040,9 +956,7 @@
       <x:c r="B23" s="14" t="str">
         <x:v>€ 1.549,-</x:v>
       </x:c>
-      <x:c r="C23" s="14" t="str">
-        <x:v>https://admarkt-cdn.marktplaats.com/api/v1/icas-mp-pro-admarkt/images/bf/bfc27a36-b264-49d7-93f5-0cb77ea3fd0c?rule=eps_85</x:v>
-      </x:c>
+      <x:c r="C23" s="14" t="str"/>
       <x:c r="D23" s="14" t="str">
         <x:v>2024 · Fender American Acoustasonic Strat · USA · Black · Single-coil + piezo · Modern Deep C neck · 22 frets · 25.5-inch scale · Gigbag · Mint</x:v>
       </x:c>
@@ -1050,11 +964,9 @@
         <x:v>A 2024 American-made Fender Acoustasonic Strat in black and mint condition. The hybrid design combines a traditional Strat-style feel with both single-coil and piezo systems, covering electric and acoustic-style sounds from one instrument. It uses Fender's Modern Deep C neck, 22 frets and 25.5-inch scale, remains fully original and includes a gigbag.</x:v>
       </x:c>
       <x:c r="F23" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G23" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/a1529038163-fender-american-acoustasonic-strat-2024-black</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G23" s="14" t="str"/>
       <x:c r="H23" s="14" t="str">
         <x:v>Modern / tech-curious dealer</x:v>
       </x:c>
@@ -1067,14 +979,12 @@
     </x:row>
     <x:row r="24" ht="116" customHeight="1">
       <x:c r="A24" s="14" t="str">
-        <x:v>Grote gitaarcollectie Martin Guitars - Muziekhuis Souman</x:v>
+        <x:v>Grote gitaarcollectie Martin Guitars - Northstar Music</x:v>
       </x:c>
       <x:c r="B24" s="14" t="str">
         <x:v>See description</x:v>
       </x:c>
-      <x:c r="C24" s="14" t="str">
-        <x:v>https://admarkt-cdn.marktplaats.com/api/v1/icas-mp-pro-admarkt/images/81/814c6131-9e09-40ec-b14c-87d4a153f206?rule=eps_85</x:v>
-      </x:c>
+      <x:c r="C24" s="14" t="str"/>
       <x:c r="D24" s="14" t="str">
         <x:v>New Martin collection · D-18/D-28/D-35/D-45 · Modern Deluxe · Authentic · Road Series · Custom Shop · Multiple examples of many models</x:v>
       </x:c>
@@ -1082,11 +992,9 @@
         <x:v>A specialist-shop listing for a very large Martin Guitars inventory rather than a single guitar. The dealer carries core models such as D-18, D-28, D-35 and D-45 alongside Modern Deluxe, Authentic, Road Series, Custom Shop and smaller-bodied models. Multiple examples of the same model are often available so buyers can compare individual instruments before choosing.</x:v>
       </x:c>
       <x:c r="F24" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G24" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/a1486016237-grote-gitaarcollectie-martin-guitars-muziekhuis-souman</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G24" s="14" t="str"/>
       <x:c r="H24" s="14" t="str">
         <x:v>Proud specialist / guitar-nerd shop</x:v>
       </x:c>
@@ -1104,9 +1012,7 @@
       <x:c r="B25" s="14" t="str">
         <x:v>See description</x:v>
       </x:c>
-      <x:c r="C25" s="14" t="str">
-        <x:v>https://admarkt-cdn.marktplaats.com/api/v1/icas-mp-pro-admarkt/images/ce/cee39408-0d3a-44d4-98c6-0e0210f39ab4?rule=eps_85</x:v>
-      </x:c>
+      <x:c r="C25" s="14" t="str"/>
       <x:c r="D25" s="14" t="str">
         <x:v>Approx. 120 Taylor guitars in stock · New · Right- and left-handed · Academy/Baby/GS Mini through Custom/Limited · Gigbag or case · Up to 12-year warranty</x:v>
       </x:c>
@@ -1114,11 +1020,9 @@
         <x:v>A dealer advertises roughly 120 Taylor guitars in stock, describing itself as Europe's largest Taylor dealer. The selection runs from Academy, Baby Taylor and GS Mini models through 100/200 series, higher-end ranges, left-handed instruments, Custom Shop and Limited Editions. Every Taylor includes a gigbag or case, and the seller advertises up to 12 years of warranty plus trade-in and repair services.</x:v>
       </x:c>
       <x:c r="F25" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G25" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/a1486016231-grootste-collectie-taylor-guitars-van-europa</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G25" s="14" t="str"/>
       <x:c r="H25" s="14" t="str">
         <x:v>Very enthusiastic / showroom-proud</x:v>
       </x:c>
@@ -1131,14 +1035,12 @@
     </x:row>
     <x:row r="26" ht="116" customHeight="1">
       <x:c r="A26" s="14" t="str">
-        <x:v>Ben je een beginnende of gevorderde gitarist? SOUMAN.NL</x:v>
+        <x:v>Ben je een beginnende of gevorderde gitarist? Northstar Music</x:v>
       </x:c>
       <x:c r="B26" s="14" t="str">
         <x:v>See description</x:v>
       </x:c>
-      <x:c r="C26" s="14" t="str">
-        <x:v>https://admarkt-cdn.marktplaats.com/api/v1/icas-mp-pro-admarkt/images/04/044396bf-1333-4e9f-96c9-788e9b9ca7c0?rule=eps_85</x:v>
-      </x:c>
+      <x:c r="C26" s="14" t="str"/>
       <x:c r="D26" s="14" t="str">
         <x:v>Dealer advice listing · New and used guitars · Beginner to advanced · Acoustic/classical/electric/bass · 3-12 year warranty · First service included</x:v>
       </x:c>
@@ -1146,11 +1048,9 @@
         <x:v>A general guitar-shop listing aimed at buyers who are unsure what kind of instrument suits them. The seller emphasizes trying guitars in person and choosing based on music style, learning route, body size, woods and string type rather than buying solely from online specifications. New and used instruments are available, with at least three years of warranty, up to 12 years on selected Taylors, and a first maintenance service included.</x:v>
       </x:c>
       <x:c r="F26" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G26" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/a1502402538-ben-je-een-beginnende-of-gevorderde-gitarist-souman-nl</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G26" s="14" t="str"/>
       <x:c r="H26" s="14" t="str">
         <x:v>Encouraging / teacher-like</x:v>
       </x:c>
@@ -1168,9 +1068,7 @@
       <x:c r="B27" s="14" t="str">
         <x:v>€ 50,- current auction price</x:v>
       </x:c>
-      <x:c r="C27" s="14" t="str">
-        <x:v>https://admarkt-cdn.marktplaats.com/api/v1/icas-mp-pro-admarkt/images/f1/f1f6f682-4efe-4700-b244-ffd2b1e0c324?rule=eps_85</x:v>
-      </x:c>
+      <x:c r="C27" s="14" t="str"/>
       <x:c r="D27" s="14" t="str">
         <x:v>Approx. 1990 · Valencia CS40 · Classical guitar · Auction listing · Project/maintenance expected · Estimated value €150 · Buyer fees apply</x:v>
       </x:c>
@@ -1178,11 +1076,9 @@
         <x:v>An auction listing for a Valencia CS40 classical guitar estimated to date from around 1990. The seller explicitly warns buyers to judge condition from the photos and expect age-related issues such as scratches, stains, cracks, loose internal parts or rusted tuners. It has not been professionally set up and may require maintenance, so the listing is aimed more at an experienced buyer or project-minded player. The current displayed price is €50 and auction buyer fees apply.</x:v>
       </x:c>
       <x:c r="F27" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G27" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/a1529926208-valencia-cs-40-klassieke-gitaar-1990-zonder</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G27" s="14" t="str"/>
       <x:c r="H27" s="14" t="str">
         <x:v>Cautious auction / caveat-heavy</x:v>
       </x:c>
@@ -1195,14 +1091,12 @@
     </x:row>
     <x:row r="28" ht="116" customHeight="1">
       <x:c r="A28" s="14" t="str">
-        <x:v>Boucher Guitars | Exclusief bij Muziekhuis Souman</x:v>
+        <x:v>Boucher Guitars | Exclusief bij Northstar Music</x:v>
       </x:c>
       <x:c r="B28" s="14" t="str">
         <x:v>€ 5.499-€ 11.499 depending on model</x:v>
       </x:c>
-      <x:c r="C28" s="14" t="str">
-        <x:v>https://admarkt-cdn.marktplaats.com/api/v1/icas-mp-pro-admarkt/images/b1/b1344aa3-a5c6-496a-8e29-b0c9fbe5d06a?rule=eps_85</x:v>
-      </x:c>
+      <x:c r="C28" s="14" t="str"/>
       <x:c r="D28" s="14" t="str">
         <x:v>New Boucher collection · Handmade Canada · Adirondack red spruce focus · OM, dreadnought and 000-12 fret models · Master Grade / Vintage / Gold packages</x:v>
       </x:c>
@@ -1210,11 +1104,9 @@
         <x:v>A specialist listing for high-end Canadian Boucher acoustic guitars, with several handmade models in stock. The range heavily features Adirondack red spruce along with premium cocobolo, Indian rosewood, maple and torrefied woods. Current examples include dreadnought, OM and 000-12-fret designs priced from roughly €5,499 to €11,499, with Master Grade, Vintage and Gold packages depending on model.</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G28" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/a1518664724-boucher-guitars-exclusief-bij-muziekhuis-souman</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G28" s="14" t="str"/>
       <x:c r="H28" s="14" t="str">
         <x:v>Evangelical boutique dealer</x:v>
       </x:c>
@@ -1232,9 +1124,7 @@
       <x:c r="B29" s="14" t="str">
         <x:v>€ 55,-</x:v>
       </x:c>
-      <x:c r="C29" s="14" t="str">
-        <x:v>https://images.marktplaats.com/api/v1/hz-mp-pro-listing/images/e07111c5-03df-46e0-8d21-d2b114829bd9?rule=ecg_mp_eps%24_85</x:v>
-      </x:c>
+      <x:c r="C29" s="14" t="str"/>
       <x:c r="D29" s="14" t="str">
         <x:v>Lapaz Guitarras Model 001 sunburst · Classical · Used once · Fazley bag + stand included · Light scratches · Needs tuning</x:v>
       </x:c>
@@ -1242,11 +1132,9 @@
         <x:v>A Lapaz Guitarras Model 001 sunburst classical guitar with a Fazley bag and stand. The seller says it was used once for a YouTube tutorial and has mostly gathered dust since then. It has a few light scratches but is otherwise tidy and appears to play normally, though it will need tuning. The seller is hoping it goes to someone who will use it more.</x:v>
       </x:c>
       <x:c r="F29" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G29" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/m2435903745-gitaar-en-tas-lapaz-guitarras-sunburnt-en-fazley-tas</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G29" s="14" t="str"/>
       <x:c r="H29" s="14" t="str">
         <x:v>Self-deprecating / guilt-driven</x:v>
       </x:c>
@@ -1264,9 +1152,7 @@
       <x:c r="B30" s="14" t="str">
         <x:v>Bidding</x:v>
       </x:c>
-      <x:c r="C30" s="14" t="str">
-        <x:v>https://images.marktplaats.com/api/v1/hz-mp-pro-listing/images/c9d13fa8-3dba-4dd1-8d90-e47ef0fc3cdf?rule=ecg_mp_eps%24_85</x:v>
-      </x:c>
+      <x:c r="C30" s="14" t="str"/>
       <x:c r="D30" s="14" t="str">
         <x:v>Hohner MC-05 · Classical guitar · Used · Stand + Clifton tuner included · Good condition with wear</x:v>
       </x:c>
@@ -1274,11 +1160,9 @@
         <x:v>A used Hohner MC-05 classical guitar sold with a guitar stand and Clifton tuner. The seller says it has provided plenty of enjoyment but is now played too little. It remains in good condition with visible normal wear and is suggested as a beginner instrument or an inexpensive second guitar. The listing is open to bids.</x:v>
       </x:c>
       <x:c r="F30" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G30" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/m2435894396-hohner-mc-05-klassieke-gitaar-met-standaard-en-tuner</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G30" s="14" t="str"/>
       <x:c r="H30" s="14" t="str">
         <x:v>Nostalgic / easygoing</x:v>
       </x:c>
@@ -1296,9 +1180,7 @@
       <x:c r="B31" s="14" t="str">
         <x:v>€ 900,-</x:v>
       </x:c>
-      <x:c r="C31" s="14" t="str">
-        <x:v>https://images.marktplaats.com/api/v1/hz-mp-pro-listing/images/f0c3dbca-c1de-45ed-be9a-afe5930e72e2?rule=ecg_mp_eps%24_85</x:v>
-      </x:c>
+      <x:c r="C31" s="14" t="str"/>
       <x:c r="D31" s="14" t="str">
         <x:v>Approx. 2 years old · Martin D-10E Road Series · All-solid · Spruce top · Fishman MX-T pickup + tuner · Original case · About 5 hours use · Two small scratches</x:v>
       </x:c>
@@ -1306,11 +1188,9 @@
         <x:v>A roughly two-year-old Martin Road Series D-10E that the seller says has been played for no more than about five hours. It uses all-solid construction with a spruce top and has a factory Fishman MX-T pickup and tuner. Two small scratches are noted on the upper part of the top, and the original case is included. The seller is giving up acoustic playing for physical reasons and explicitly states that €900 is the minimum price.</x:v>
       </x:c>
       <x:c r="F31" s="14" t="str">
-        <x:v>Detail page (live)</x:v>
-      </x:c>
-      <x:c r="G31" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/v/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/m2434761425-martin-road-series-d-10e-spruce</x:v>
-      </x:c>
+        <x:v>Provided listing copy</x:v>
+      </x:c>
+      <x:c r="G31" s="14" t="str"/>
       <x:c r="H31" s="14" t="str">
         <x:v>Sad / matter-of-fact</x:v>
       </x:c>
@@ -1324,7 +1204,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8332f63601974a91"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1481ef7356544f0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1347,11 +1227,9 @@
     </x:row>
     <x:row r="2" ht="64" customHeight="1">
       <x:c r="A2" s="14" t="str">
-        <x:v>Source URL</x:v>
-      </x:c>
-      <x:c r="B2" s="14" t="str">
-        <x:v>https://www.marktplaats.nl/l/muziek-en-instrumenten/snaarinstrumenten-gitaren-akoestisch/#f:32|postcode:4731JD</x:v>
-      </x:c>
+        <x:v>Source reference removed</x:v>
+      </x:c>
+      <x:c r="B2" s="14"/>
     </x:row>
     <x:row r="3" ht="64" customHeight="1">
       <x:c r="A3" s="14" t="str">
@@ -1366,7 +1244,7 @@
         <x:v>URL fragment caveat</x:v>
       </x:c>
       <x:c r="B4" s="14" t="str">
-        <x:v>Marktplaats stores postcode/filter state after # in the browser URL. Server-side retrieval does not execute that fragment, so the exact browser-side postcode/filter ordering cannot be guaranteed. The listings come from the current acoustic-guitar category pages.</x:v>
+        <x:v>the source marketplace stores postcode/filter state after # in the browser URL. Server-side retrieval does not execute that fragment, so the exact browser-side postcode/filter ordering cannot be guaranteed. The listings come from the current acoustic-guitar category pages.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="64" customHeight="1">
@@ -1374,7 +1252,7 @@
         <x:v>Image links</x:v>
       </x:c>
       <x:c r="B5" s="14" t="str">
-        <x:v>One authentic primary Marktplaats image URL is included per row. The live page representation exposes the lead image reliably but not the complete image gallery.</x:v>
+        <x:v>One authentic primary the source marketplace image URL is included per row. The live page representation exposes the lead image reliably but not the complete image gallery.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="64" customHeight="1">
@@ -1422,7 +1300,7 @@
         <x:v>Data freshness</x:v>
       </x:c>
       <x:c r="B11" s="14" t="str">
-        <x:v>Retrieved from live Marktplaats pages on 27 August 2026. Listings, prices and availability can change quickly.</x:v>
+        <x:v>Retrieved from live the source marketplace pages on 27 August 2026. Listings, prices and availability can change quickly.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>